<commit_message>
Updates to design docs. Added vivado/scripts/reset_and_synth.tcl. Added multicycle path constraints to angus.xdc
</commit_message>
<xml_diff>
--- a/docs/Pi Header Pin Mapping.xlsx
+++ b/docs/Pi Header Pin Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\f402n\Desktop\yocto_shared\Angus\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C764A06-50AD-4689-AB73-A40BAB20B61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F302CA50-3036-4CDB-AA88-BF32860AEA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37350" yWindow="3030" windowWidth="16740" windowHeight="18780" xr2:uid="{5C3ACEC7-C3F8-4CFC-A1B6-03B295AD6612}"/>
+    <workbookView xWindow="4305" yWindow="1290" windowWidth="28845" windowHeight="19710" xr2:uid="{5C3ACEC7-C3F8-4CFC-A1B6-03B295AD6612}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="151">
   <si>
     <t>Pi Header Pin Number</t>
   </si>
@@ -371,9 +371,6 @@
     <t>Clk Pins</t>
   </si>
   <si>
-    <t>crank_signal_ok</t>
-  </si>
-  <si>
     <t>sync_full</t>
   </si>
   <si>
@@ -431,20 +428,77 @@
     <t>phase_ref_found</t>
   </si>
   <si>
-    <t>crank_ab_edge</t>
-  </si>
-  <si>
     <t>ab_edge</t>
   </si>
   <si>
     <t>z_edge</t>
+  </si>
+  <si>
+    <t>D0</t>
+  </si>
+  <si>
+    <t>Scope Ch</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>D8</t>
+  </si>
+  <si>
+    <t>D9</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>D13</t>
+  </si>
+  <si>
+    <t>D14</t>
+  </si>
+  <si>
+    <t>D15</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>crank_ab</t>
+  </si>
+  <si>
+    <t>crank_sig_ok</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -460,8 +514,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -471,6 +538,54 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC9900"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9900"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -487,7 +602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -505,12 +620,42 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF9900"/>
+      <color rgb="FFCC9900"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -839,7 +984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7434CF07-7DD9-4123-945B-957DE6235948}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -849,9 +994,10 @@
     <col min="5" max="5" width="18.5703125" style="3" customWidth="1"/>
     <col min="6" max="6" width="9.140625" style="3"/>
     <col min="7" max="7" width="17.28515625" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -873,8 +1019,12 @@
       <c r="G1" s="2" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L1" s="2"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -882,7 +1032,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -891,7 +1041,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -910,8 +1060,11 @@
       <c r="G4" s="3" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I4" s="7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -919,7 +1072,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -938,16 +1091,22 @@
       <c r="G6" s="3" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I6" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I7" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -964,10 +1123,13 @@
         <v>101</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -981,13 +1143,16 @@
         <v>5</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -995,7 +1160,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1012,7 +1177,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1029,7 +1194,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1046,10 +1211,13 @@
         <v>92</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1066,7 +1234,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1074,7 +1242,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1091,10 +1259,13 @@
         <v>99</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1111,18 +1282,27 @@
         <v>98</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="L17" s="12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L18" s="13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1139,7 +1319,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1156,10 +1336,13 @@
         <v>93</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1167,7 +1350,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1181,13 +1364,16 @@
         <v>68</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1201,10 +1387,10 @@
         <v>78</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1221,10 +1407,13 @@
         <v>95</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1238,10 +1427,10 @@
         <v>77</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1249,7 +1438,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1263,10 +1452,10 @@
         <v>90</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1280,10 +1469,10 @@
         <v>86</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1297,10 +1486,10 @@
         <v>87</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1317,10 +1506,13 @@
         <v>100</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1328,7 +1520,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1342,10 +1534,10 @@
         <v>89</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -1362,10 +1554,13 @@
         <v>97</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1382,18 +1577,24 @@
         <v>96</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I35" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -1410,7 +1611,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -1427,10 +1628,13 @@
         <v>94</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -1444,10 +1648,10 @@
         <v>75</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -1461,18 +1665,21 @@
         <v>82</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I40" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -1489,12 +1696,13 @@
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E43" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Unit tests working again.
Debugged crank and cam on hardware. Phase partly working, needs further debugging of raw_phase and phase_eng.
Improved reset_and_build.tcl script to rebuild after changed hdl files without GUI interaction.
</commit_message>
<xml_diff>
--- a/docs/Pi Header Pin Mapping.xlsx
+++ b/docs/Pi Header Pin Mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\f402n\Desktop\yocto_shared\Angus\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F302CA50-3036-4CDB-AA88-BF32860AEA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D6E353-40AA-4F2B-B024-C5FB8C5D477E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4305" yWindow="1290" windowWidth="28845" windowHeight="19710" xr2:uid="{5C3ACEC7-C3F8-4CFC-A1B6-03B295AD6612}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="146">
   <si>
     <t>Pi Header Pin Number</t>
   </si>
@@ -374,124 +374,109 @@
     <t>sync_full</t>
   </si>
   <si>
+    <t>trig_pulse</t>
+  </si>
+  <si>
+    <t>debug_out_0[12]</t>
+  </si>
+  <si>
+    <t>debug_out_0[13]</t>
+  </si>
+  <si>
+    <t>debug_out_0[14]</t>
+  </si>
+  <si>
+    <t>debug_out_0[15]</t>
+  </si>
+  <si>
+    <t>phase_inv_latch</t>
+  </si>
+  <si>
+    <t>phase_ref_found</t>
+  </si>
+  <si>
+    <t>z_edge</t>
+  </si>
+  <si>
+    <t>D0</t>
+  </si>
+  <si>
+    <t>Scope Ch</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>D8</t>
+  </si>
+  <si>
+    <t>D9</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>D11</t>
+  </si>
+  <si>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>D13</t>
+  </si>
+  <si>
+    <t>D14</t>
+  </si>
+  <si>
+    <t>D15</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>crank_ab</t>
+  </si>
+  <si>
+    <t>crank_z</t>
+  </si>
+  <si>
+    <t>ref_det</t>
+  </si>
+  <si>
+    <t>crank_gap_det</t>
+  </si>
+  <si>
+    <t>ab_edge</t>
+  </si>
+  <si>
+    <t>cam_edge</t>
+  </si>
+  <si>
     <t>ref_edge</t>
   </si>
   <si>
-    <t>crank_gap_get</t>
-  </si>
-  <si>
-    <t>phase_ref_det</t>
-  </si>
-  <si>
-    <t>trig_pulse</t>
-  </si>
-  <si>
-    <t>pll_div_valid</t>
-  </si>
-  <si>
-    <t>debug_out_0[12]</t>
-  </si>
-  <si>
-    <t>debug_out_0[13]</t>
-  </si>
-  <si>
-    <t>debug_out_0[14]</t>
-  </si>
-  <si>
-    <t>debug_out_0[15]</t>
-  </si>
-  <si>
-    <t>debug_out_0[16]</t>
-  </si>
-  <si>
-    <t>debug_out_0[17]</t>
-  </si>
-  <si>
-    <t>debug_out_0[18]</t>
-  </si>
-  <si>
-    <t>debug_out_0[19]</t>
-  </si>
-  <si>
-    <t>debug_out_0[20]</t>
-  </si>
-  <si>
-    <t>debug_out_0[21]</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> =not yet implemented</t>
-  </si>
-  <si>
-    <t>phase_inv_latch</t>
-  </si>
-  <si>
-    <t>phase_ref_found</t>
-  </si>
-  <si>
-    <t>ab_edge</t>
-  </si>
-  <si>
-    <t>z_edge</t>
-  </si>
-  <si>
-    <t>D0</t>
-  </si>
-  <si>
-    <t>Scope Ch</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>D2</t>
-  </si>
-  <si>
-    <t>D3</t>
-  </si>
-  <si>
-    <t>D4</t>
-  </si>
-  <si>
-    <t>D5</t>
-  </si>
-  <si>
-    <t>D6</t>
-  </si>
-  <si>
-    <t>D7</t>
-  </si>
-  <si>
-    <t>D8</t>
-  </si>
-  <si>
-    <t>D9</t>
-  </si>
-  <si>
-    <t>D10</t>
-  </si>
-  <si>
-    <t>D11</t>
-  </si>
-  <si>
-    <t>D12</t>
-  </si>
-  <si>
-    <t>D13</t>
-  </si>
-  <si>
-    <t>D14</t>
-  </si>
-  <si>
-    <t>D15</t>
-  </si>
-  <si>
-    <t>GND</t>
-  </si>
-  <si>
-    <t>crank_ab</t>
-  </si>
-  <si>
-    <t>crank_sig_ok</t>
+    <t>phase_raw</t>
+  </si>
+  <si>
+    <t>phase_eng</t>
   </si>
 </sst>
 </file>
@@ -617,9 +602,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -638,10 +620,13 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1020,7 +1005,7 @@
         <v>107</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="L1" s="2"/>
     </row>
@@ -1060,8 +1045,8 @@
       <c r="G4" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>131</v>
+      <c r="I4" s="6" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1089,10 +1074,10 @@
         <v>102</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>133</v>
+        <v>140</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1102,8 +1087,8 @@
       <c r="B7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="14" t="s">
-        <v>148</v>
+      <c r="I7" s="12" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1123,10 +1108,10 @@
         <v>101</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>134</v>
+        <v>137</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1143,13 +1128,13 @@
         <v>5</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1208,14 +1193,15 @@
         <v>79</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>110</v>
+        <v>141</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>144</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="K13" s="3"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
@@ -1256,16 +1242,16 @@
         <v>66</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1279,30 +1265,24 @@
         <v>70</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="I17" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="L17" s="12" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L18" s="13" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1319,7 +1299,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1333,24 +1313,27 @@
         <v>67</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I21" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1364,16 +1347,16 @@
         <v>68</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="G22" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="I22" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="I22" s="8" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1386,11 +1369,18 @@
       <c r="D23" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E23" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E23" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1404,16 +1394,17 @@
         <v>69</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I24" s="11" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1426,11 +1417,17 @@
       <c r="D25" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E25" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1438,7 +1435,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1451,11 +1448,17 @@
       <c r="D27" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E27" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1468,11 +1471,17 @@
       <c r="D28" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E28" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1485,11 +1494,17 @@
       <c r="D29" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E29" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1503,16 +1518,16 @@
         <v>88</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>111</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1520,7 +1535,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1532,9 +1547,6 @@
       </c>
       <c r="D32" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -1550,15 +1562,7 @@
       <c r="D33" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>136</v>
-      </c>
+      <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
@@ -1573,15 +1577,7 @@
       <c r="D34" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="I34" s="14" t="s">
-        <v>140</v>
-      </c>
+      <c r="G34" s="3"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
@@ -1590,8 +1586,8 @@
       <c r="B35" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I35" s="14" t="s">
-        <v>148</v>
+      <c r="I35" s="12" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -1624,15 +1620,7 @@
       <c r="D37" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="I37" s="10" t="s">
-        <v>143</v>
-      </c>
+      <c r="G37" s="3"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
@@ -1647,9 +1635,6 @@
       <c r="D38" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E38" s="5" t="s">
-        <v>124</v>
-      </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
@@ -1664,9 +1649,6 @@
       <c r="D39" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E39" s="5" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
@@ -1675,8 +1657,8 @@
       <c r="B40" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I40" s="14" t="s">
-        <v>148</v>
+      <c r="I40" s="12" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -1697,9 +1679,7 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E43" s="6" t="s">
-        <v>126</v>
-      </c>
+      <c r="E43" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Adjusted design docs to v3 before refactoring
</commit_message>
<xml_diff>
--- a/docs/Pi Header Pin Mapping.xlsx
+++ b/docs/Pi Header Pin Mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\f402n\Desktop\yocto_shared\Angus\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D6E353-40AA-4F2B-B024-C5FB8C5D477E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A240349-18A6-4B79-A89A-AE8F2F6DB244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4305" yWindow="1290" windowWidth="28845" windowHeight="19710" xr2:uid="{5C3ACEC7-C3F8-4CFC-A1B6-03B295AD6612}"/>
+    <workbookView xWindow="-29760" yWindow="-11250" windowWidth="28845" windowHeight="19710" xr2:uid="{5C3ACEC7-C3F8-4CFC-A1B6-03B295AD6612}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="144">
   <si>
     <t>Pi Header Pin Number</t>
   </si>
@@ -374,9 +374,6 @@
     <t>sync_full</t>
   </si>
   <si>
-    <t>trig_pulse</t>
-  </si>
-  <si>
     <t>debug_out_0[12]</t>
   </si>
   <si>
@@ -389,9 +386,6 @@
     <t>debug_out_0[15]</t>
   </si>
   <si>
-    <t>phase_inv_latch</t>
-  </si>
-  <si>
     <t>phase_ref_found</t>
   </si>
   <si>
@@ -473,10 +467,10 @@
     <t>ref_edge</t>
   </si>
   <si>
-    <t>phase_raw</t>
-  </si>
-  <si>
     <t>phase_eng</t>
+  </si>
+  <si>
+    <t>trig_edge</t>
   </si>
 </sst>
 </file>
@@ -1005,7 +999,7 @@
         <v>107</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="L1" s="2"/>
     </row>
@@ -1046,7 +1040,7 @@
         <v>105</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1074,10 +1068,10 @@
         <v>102</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1088,7 +1082,7 @@
         <v>10</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1108,10 +1102,10 @@
         <v>101</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1131,10 +1125,10 @@
         <v>100</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1196,10 +1190,10 @@
         <v>99</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K13" s="3"/>
     </row>
@@ -1245,10 +1239,10 @@
         <v>98</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1271,7 +1265,7 @@
         <v>106</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1316,10 +1310,10 @@
         <v>96</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -1330,7 +1324,7 @@
         <v>10</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1350,10 +1344,10 @@
         <v>95</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1373,10 +1367,10 @@
         <v>94</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K23" s="3"/>
     </row>
@@ -1397,10 +1391,10 @@
         <v>93</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K24" s="3"/>
     </row>
@@ -1421,10 +1415,10 @@
         <v>92</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1449,13 +1443,13 @@
         <v>90</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -1472,13 +1466,13 @@
         <v>86</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1495,13 +1489,10 @@
         <v>87</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -1518,13 +1509,10 @@
         <v>88</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1587,7 +1575,7 @@
         <v>10</v>
       </c>
       <c r="I35" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -1658,7 +1646,7 @@
         <v>10</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>